<commit_message>
:bar_chart: feat(excel): inclusão de conceitos sobre células e intervalos
</commit_message>
<xml_diff>
--- a/myFirstWorkbook.xlsx
+++ b/myFirstWorkbook.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nitro5\OneDrive\Documentos\GitHub\Bootcamp-DIO-Bradesco-GenAI-Dados\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A8F5C4-7171-44A4-846B-8FFA7FF3ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="18180" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,8 +24,37 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>Célula (Cell)</t>
+  </si>
+  <si>
+    <t>Intervalo (range) - Conjunto de células selecionadas</t>
+  </si>
+  <si>
+    <t>D6 : G6</t>
+  </si>
+  <si>
+    <t>Seleção do intervalo inteiro de células</t>
+  </si>
+  <si>
+    <t>D6 ; G6</t>
+  </si>
+  <si>
+    <t>Seleção do intervalo de células específicas</t>
+  </si>
+  <si>
+    <t>D1:D3 ; G1:G3</t>
+  </si>
+  <si>
+    <t>Combinação de intervalos</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -29,12 +64,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +90,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +372,52 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="B2:F8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
:bar_chart: feat(excel): aplicação da função ALEATÓRIOENTRE e atalhos de produtividade
</commit_message>
<xml_diff>
--- a/myFirstWorkbook.xlsx
+++ b/myFirstWorkbook.xlsx
@@ -5,27 +5,39 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nitro5\OneDrive\Documentos\GitHub\Bootcamp-DIO-Bradesco-GenAI-Dados\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17070c8bd82a19a8/Documentos/GitHub/Bootcamp-DIO-Bradesco-GenAI-Dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A8F5C4-7171-44A4-846B-8FFA7FF3ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{93A8F5C4-7171-44A4-846B-8FFA7FF3ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A066F990-740C-4EDF-BA42-82A01640867B}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="18180" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="17655" yWindow="0" windowWidth="11250" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="aula2" sheetId="1" r:id="rId1"/>
+    <sheet name="aula4" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Célula (Cell)</t>
   </si>
@@ -49,14 +61,46 @@
   </si>
   <si>
     <t>Combinação de intervalos</t>
+  </si>
+  <si>
+    <t>loja</t>
+  </si>
+  <si>
+    <t>valor de venda</t>
+  </si>
+  <si>
+    <t>loja a</t>
+  </si>
+  <si>
+    <t>loja b</t>
+  </si>
+  <si>
+    <t>loja c</t>
+  </si>
+  <si>
+    <t>selecionar o intervalo &gt; apertar F2 &gt; apertar ctrl+enter</t>
+  </si>
+  <si>
+    <t>uso da formula ALEATÓRIOENTRE</t>
+  </si>
+  <si>
+    <t>copiado a seleção e colado como valores utiliando ctrl+alt+v</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -90,9 +134,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -420,4 +465,58 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26EE5D11-5C86-4A55-BEBE-6D3C447EC4BD}">
+  <dimension ref="B2:E5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>108</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <v>205</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5">
+        <v>327</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
:bar_chart: feat(excel): estudo sobre congelamento de células e uso do atalho F4
</commit_message>
<xml_diff>
--- a/myFirstWorkbook.xlsx
+++ b/myFirstWorkbook.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17070c8bd82a19a8/Documentos/GitHub/Bootcamp-DIO-Bradesco-GenAI-Dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{93A8F5C4-7171-44A4-846B-8FFA7FF3ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A066F990-740C-4EDF-BA42-82A01640867B}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{93A8F5C4-7171-44A4-846B-8FFA7FF3ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85B504C1-F4FA-4574-B7D4-7BAAEE4569C8}"/>
   <bookViews>
-    <workbookView xWindow="17655" yWindow="0" windowWidth="11250" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aula2" sheetId="1" r:id="rId1"/>
     <sheet name="aula4" sheetId="2" r:id="rId2"/>
+    <sheet name="aula5" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
   <si>
     <t>Célula (Cell)</t>
   </si>
@@ -85,6 +86,18 @@
   </si>
   <si>
     <t>copiado a seleção e colado como valores utiliando ctrl+alt+v</t>
+  </si>
+  <si>
+    <t>congelamento de celulas</t>
+  </si>
+  <si>
+    <t>congelado</t>
+  </si>
+  <si>
+    <t>não congelado</t>
+  </si>
+  <si>
+    <t>usando $$ para congelar linhas e colunas (atalho F4)</t>
   </si>
 </sst>
 </file>
@@ -153,6 +166,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -519,4 +536,87 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{753BAFF7-ECC7-4397-9E88-3D628CF658CC}">
+  <dimension ref="B2:G5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <v>108</v>
+      </c>
+      <c r="D3">
+        <f>SUM($C$3:C3)</f>
+        <v>108</v>
+      </c>
+      <c r="E3">
+        <f>SUM(C3:C3)</f>
+        <v>108</v>
+      </c>
+      <c r="G3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4">
+        <v>205</v>
+      </c>
+      <c r="D4">
+        <f>SUM($C$3:C4)</f>
+        <v>313</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E5" si="0">SUM(C4:C4)</f>
+        <v>205</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5">
+        <v>327</v>
+      </c>
+      <c r="D5">
+        <f>SUM($C$3:C5)</f>
+        <v>640</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>327</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
:bar_chart: feat(excel): formatação, validação de dados, fórmulas de contagem e gráfico de progresso
</commit_message>
<xml_diff>
--- a/myFirstWorkbook.xlsx
+++ b/myFirstWorkbook.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17070c8bd82a19a8/Documentos/GitHub/Bootcamp-DIO-Bradesco-GenAI-Dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{93A8F5C4-7171-44A4-846B-8FFA7FF3ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{85B504C1-F4FA-4574-B7D4-7BAAEE4569C8}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="13_ncr:1_{93A8F5C4-7171-44A4-846B-8FFA7FF3ACC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF42F93C-88B7-43C1-8FAC-C949095B0B1E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aula2" sheetId="1" r:id="rId1"/>
     <sheet name="aula4" sheetId="2" r:id="rId2"/>
     <sheet name="aula5" sheetId="3" r:id="rId3"/>
+    <sheet name="Prática" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
   <si>
     <t>Célula (Cell)</t>
   </si>
@@ -98,13 +99,58 @@
   </si>
   <si>
     <t>usando $$ para congelar linhas e colunas (atalho F4)</t>
+  </si>
+  <si>
+    <t>Backlog</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Orçamentos Ball</t>
+  </si>
+  <si>
+    <t>Planilha caracteristicas painéis</t>
+  </si>
+  <si>
+    <t>Laís</t>
+  </si>
+  <si>
+    <t>Done</t>
+  </si>
+  <si>
+    <t>Working</t>
+  </si>
+  <si>
+    <t>Criar Skyrim Books App</t>
+  </si>
+  <si>
+    <t>Stuck</t>
+  </si>
+  <si>
+    <t>Total de Atividades:</t>
+  </si>
+  <si>
+    <t>Atividades Concluidas:</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -120,8 +166,42 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Segoe UI Light"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI Light"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -134,8 +214,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -143,20 +241,91 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color theme="0"/>
+      </left>
+      <right style="thick">
+        <color theme="0"/>
+      </right>
+      <top style="thick">
+        <color theme="0"/>
+      </top>
+      <bottom style="thick">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Título 2" xfId="1" builtinId="17"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF92D050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDE445A"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFDE445A"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -166,6 +335,861 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="pt-BR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0"/>
+          <c:y val="0.22083779250732305"/>
+          <c:w val="0.9910700505315605"/>
+          <c:h val="0.5583244149853539"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prática!$I$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Total de Atividades:</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="bg2">
+                  <a:lumMod val="90000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-E6D3-440D-9F8A-6ADA564756B9}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:val>
+            <c:numRef>
+              <c:f>Prática!$J$4</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-E6D3-440D-9F8A-6ADA564756B9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="308646352"/>
+        <c:axId val="308645872"/>
+      </c:barChart>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="stacked"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Prática!$I$5</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Atividades Concluidas:</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="92D050"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>Prática!$J$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-E6D3-440D-9F8A-6ADA564756B9}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="150"/>
+        <c:overlap val="100"/>
+        <c:axId val="480098752"/>
+        <c:axId val="480099712"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="308646352"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="308645872"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="308645872"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="308646352"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="480099712"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="t"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="480098752"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="480098752"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="l"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="480099712"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="25400">
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:noFill/>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="pt-BR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.78740157499999996" l="0.511811024" r="0.511811024" t="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="297">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>584639</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>103133</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>164224</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>190501</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27AE9015-3953-0EF1-2F2A-465D89E3F8B7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -619,4 +1643,209 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB3139C4-1AEF-4B02-9D0E-3781438C7688}">
+  <dimension ref="B1:J15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="2.7109375" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="8.7109375" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" customWidth="1"/>
+    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:10" s="3" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:10" s="8" customFormat="1" ht="57.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="3" spans="2:10" s="10" customFormat="1" ht="24" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B3" s="9"/>
+      <c r="C3" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="5"/>
+      <c r="C4" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="12">
+        <v>46097</v>
+      </c>
+      <c r="G4" s="11">
+        <v>3</v>
+      </c>
+      <c r="I4" t="s">
+        <v>33</v>
+      </c>
+      <c r="J4">
+        <f>COUNTA(C4:C13)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="5"/>
+      <c r="C5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="12">
+        <v>46111</v>
+      </c>
+      <c r="G5" s="11">
+        <v>1</v>
+      </c>
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5">
+        <f>COUNTIF(E4:E13,"Done")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="5"/>
+      <c r="C6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="12">
+        <v>46351</v>
+      </c>
+      <c r="G6" s="11">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="5"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+    </row>
+    <row r="8" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="5"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+    </row>
+    <row r="9" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="5"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+    </row>
+    <row r="10" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="5"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+    </row>
+    <row r="11" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="5"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+    </row>
+    <row r="12" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="5"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+    </row>
+    <row r="13" spans="2:10" ht="15.95" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="5"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+    </row>
+    <row r="14" spans="2:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H15" s="4"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E4:E13">
+    <cfRule type="expression" dxfId="2" priority="2">
+      <formula>$E4="Stuck"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="3">
+      <formula>$E4="Working"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>$E4="Done"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G13">
+    <cfRule type="iconSet" priority="1">
+      <iconSet iconSet="4Rating" showValue="0">
+        <cfvo type="percent" val="0"/>
+        <cfvo type="num" val="2"/>
+        <cfvo type="num" val="3"/>
+        <cfvo type="num" val="4"/>
+      </iconSet>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E4:E13" xr:uid="{F7BC2505-59FB-402E-8D0D-D17C63D5918E}">
+      <formula1>"Stuck,Working,Done"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>